<commit_message>
- minimale Datenblatt und BOM Korrekturen
</commit_message>
<xml_diff>
--- a/BOM/20211104 BOM TeKaDe Baseboard.xlsx
+++ b/BOM/20211104 BOM TeKaDe Baseboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\PCB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A1FBD8-9BCD-43D0-AB9A-4854D169AC6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF00EC4-94E6-493E-A50F-8D7577B16A1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11960" xr2:uid="{261E8F2A-9F01-4E4B-AED6-14B6866C8B8C}"/>
   </bookViews>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="52" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" s="40" t="s">
         <v>251</v>

</xml_diff>